<commit_message>
Complete tasks 20-23: stagger each/amount to distribute()
</commit_message>
<xml_diff>
--- a/gsap_self_study.xlsx
+++ b/gsap_self_study.xlsx
@@ -2308,9 +2308,21 @@
           <t>04-stagger</t>
         </is>
       </c>
-      <c r="Q21" s="4" t="n"/>
-      <c r="R21" s="4" t="n"/>
-      <c r="S21" s="4" t="n"/>
+      <c r="Q21" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="R21" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="S21" s="4" t="inlineStr">
+        <is>
+          <t>Version A = stagger: { amount: 1 } -&gt; TOTAL spread of start times is 1s so the 5th and the 50th box both START at the 1s mark (gap = 1/(n-1)). Version B = stagger: { each: 0.1 } -&gt; FIXED gap per item so 5 items = 0.4s wave, 50 items = 4.9s. A bare number (stagger: 0.1) is shorthand for each. Proved with a count state (5 / 50 buttons) + dependencies: [count] on useGSAP so the tween re-runs on the new boxes. Used gsap.fromTo (explicit start y:-100 autoAlpha:0) because 50 -&gt; 5 reuses the first five DOM nodes which already sit at the end values - gsap.to had nowhere to go. Stagger gap != tween duration: each item still takes its own 0.5s.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -2385,9 +2397,21 @@
           <t>04-stagger</t>
         </is>
       </c>
-      <c r="Q22" s="4" t="n"/>
-      <c r="R22" s="4" t="n"/>
-      <c r="S22" s="4" t="n"/>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="R22" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="S22" s="4" t="inlineStr">
+        <is>
+          <t>Ripple: row of 15 dots; click handler wrapped in contextSafe (config-only useGSAP({ scope }) is valid when there is no mount tween - ONE call per component is the rule). gsap.to('.box' { scale: 0.1 repeat: 1 yoyo: true stagger: { from: index amount: 1 ease } }) - from: &lt;index&gt; makes the clicked dot start first and the wave spreads BOTH ways; from: 'center' / 'edges' / 'start' are the named origins. yoyo needs repeat or the dots just shrink and stay. amount: 1 keeps the whole ripple at 1s from any origin. Stagger ease (inside the stagger object) shapes the GAPS between start times; the tween ease shapes each dot's own motion - two separate clocks. axis only matters with grid (lesson 22). overwrite: 'auto' (lowercase) stops rapid clicks stacking scale tweens.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -2462,9 +2486,21 @@
           <t>04-stagger</t>
         </is>
       </c>
-      <c r="Q23" s="4" t="n"/>
-      <c r="R23" s="4" t="n"/>
-      <c r="S23" s="4" t="n"/>
+      <c r="Q23" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="R23" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="S23" s="4" t="inlineStr">
+        <is>
+          <t>10x10 tile wall (Array.from 100 + grid-cols-10) so DOM order = visual rows. Same handler shape as lab 21 (contextSafe, from: index, amount: 1, repeat 1 + yoyo, overwrite 'auto' lowercase). grid: [10, 10] (rows, cols; or 'auto' = GSAP measures the layout) makes from: index mean 'the tile at that grid position' and every other tile's delay = straight-line distance from it -&gt; ring from the centre, quarter-circle from a corner, far corner last, diagonal arrives with the straight lines. Without grid the same from: index snakes row by row in DOM order. axis: 'x' = distance measured horizontally only -&gt; the clicked COLUMN moves first and the wave sweeps left/right; axis: 'y' = row sweep. axis is ignored without grid. Verified circle + corner; axis variant tested by toggling the key (left commented for the 2D default).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2535,9 +2571,21 @@
         <v>1</v>
       </c>
       <c r="P24" s="3" t="n"/>
-      <c r="Q24" s="4" t="n"/>
-      <c r="R24" s="4" t="n"/>
-      <c r="S24" s="4" t="n"/>
+      <c r="Q24" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="R24" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="S24" s="4" t="inlineStr">
+        <is>
+          <t>Fan of 7 absolute cards (relative wrapper, origin-bottom) from ONE gsap.to('.card'). distribute returns a FUNCTION (i, target, arr) -&gt; value; pass the function itself as the property value - GSAP calls it per card. Config keys: base, amount, each, from, ease, grid, axis (there is NO end). base = value at the from position, base + amount = value at the farthest card, so -30 to 30 = base -30 amount 60 (default from start). from: 'center' hands BASE to the middle card so with base 0.9 the centre was the SMALLEST - fixed with from: 'edges' (edges get base, centre gets base + amount). Stagger amount: 1 unfolds the fan; replay = stored tween in a ref + play/reverse toggle (steer only, no contextSafe). Changing 7 -&gt; 9 still fans evenly with no code change. 'random(-30,30)' = scatter (unrelated per-card values), distribute = evenly SPACED values.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">

</xml_diff>